<commit_message>
Agrega parametro Corriente de fuga (mA) en puesta a tierra
- Nueva columna 'Corriente de fuga (mA)' en cada hoja de equipo del
  Excel, justo despues de Resistencia tierra (datos sinteticos de
  ejemplo, correlacionados con la resistencia de tierra).
- COLUMNAS de agente.py incluye el parametro (monitoreo, sin limite).
- reporte_completo lo muestra en la seccion de puesta a tierra.
- README documenta el parametro y como clasificarlo si se desea.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Mantenimiento_Subestaciones.xlsx
+++ b/Mantenimiento_Subestaciones.xlsx
@@ -516,11 +516,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
     <col width="42" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
@@ -552,35 +553,40 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Corriente de fuga (mA)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Corriente Fase A (A)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Corriente Fase B (A)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Corriente Fase C (A)</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Potencia Activa (MW)</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Potencia Reactiva (MVAR)</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Num Operaciones</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Observacion</t>
         </is>
@@ -607,21 +613,24 @@
         <v>2.1</v>
       </c>
       <c r="F2" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="G2" t="n">
         <v>114.7</v>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>116.4</v>
       </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
         <v>117.5</v>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>6.23</v>
       </c>
-      <c r="J2" t="n">
+      <c r="K2" t="n">
         <v>3.07</v>
       </c>
-      <c r="K2" t="n">
+      <c r="L2" t="n">
         <v>3408</v>
       </c>
     </row>
@@ -646,21 +655,24 @@
         <v>3.7</v>
       </c>
       <c r="F3" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="G3" t="n">
         <v>93.8</v>
-      </c>
-      <c r="G3" t="n">
-        <v>92.40000000000001</v>
       </c>
       <c r="H3" t="n">
         <v>92.40000000000001</v>
       </c>
       <c r="I3" t="n">
+        <v>92.40000000000001</v>
+      </c>
+      <c r="J3" t="n">
         <v>4.97</v>
       </c>
-      <c r="J3" t="n">
+      <c r="K3" t="n">
         <v>2.46</v>
       </c>
-      <c r="K3" t="n">
+      <c r="L3" t="n">
         <v>10711</v>
       </c>
     </row>
@@ -685,21 +697,24 @@
         <v>4.6</v>
       </c>
       <c r="F4" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="G4" t="n">
         <v>79</v>
-      </c>
-      <c r="G4" t="n">
-        <v>79.59999999999999</v>
       </c>
       <c r="H4" t="n">
         <v>79.59999999999999</v>
       </c>
       <c r="I4" t="n">
+        <v>79.59999999999999</v>
+      </c>
+      <c r="J4" t="n">
         <v>4.3</v>
       </c>
-      <c r="J4" t="n">
+      <c r="K4" t="n">
         <v>2</v>
       </c>
-      <c r="K4" t="n">
+      <c r="L4" t="n">
         <v>7737</v>
       </c>
     </row>
@@ -724,24 +739,27 @@
         <v>2.3</v>
       </c>
       <c r="F5" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="G5" t="n">
         <v>84.90000000000001</v>
       </c>
-      <c r="G5" t="n">
+      <c r="H5" t="n">
         <v>93.5</v>
       </c>
-      <c r="H5" t="n">
+      <c r="I5" t="n">
         <v>122.3</v>
       </c>
-      <c r="I5" t="n">
+      <c r="J5" t="n">
         <v>5.31</v>
       </c>
-      <c r="J5" t="n">
+      <c r="K5" t="n">
         <v>2.77</v>
       </c>
-      <c r="K5" t="n">
+      <c r="L5" t="n">
         <v>9359</v>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>Desbalance de corrientes entre fases</t>
         </is>
@@ -763,11 +781,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
     <col width="42" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
@@ -799,35 +818,40 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Corriente de fuga (mA)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Corriente Fase A (A)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Corriente Fase B (A)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Corriente Fase C (A)</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Potencia Activa (MW)</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Potencia Reactiva (MVAR)</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Num Operaciones</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Observacion</t>
         </is>
@@ -854,21 +878,24 @@
         <v>3.5</v>
       </c>
       <c r="F2" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="G2" t="n">
         <v>78.09999999999999</v>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>79</v>
       </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
         <v>78.3</v>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>4.34</v>
       </c>
-      <c r="J2" t="n">
+      <c r="K2" t="n">
         <v>1.76</v>
       </c>
-      <c r="K2" t="n">
+      <c r="L2" t="n">
         <v>3013</v>
       </c>
     </row>
@@ -893,24 +920,27 @@
         <v>4.5</v>
       </c>
       <c r="F3" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="G3" t="n">
         <v>91.7</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>84.90000000000001</v>
       </c>
-      <c r="H3" t="n">
+      <c r="I3" t="n">
         <v>80.8</v>
       </c>
-      <c r="I3" t="n">
+      <c r="J3" t="n">
         <v>4.83</v>
       </c>
-      <c r="J3" t="n">
+      <c r="K3" t="n">
         <v>1.72</v>
       </c>
-      <c r="K3" t="n">
+      <c r="L3" t="n">
         <v>3341</v>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>Desbalance de corrientes entre fases</t>
         </is>
@@ -937,21 +967,24 @@
         <v>2.2</v>
       </c>
       <c r="F4" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="G4" t="n">
         <v>79.09999999999999</v>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>80.2</v>
       </c>
-      <c r="H4" t="n">
+      <c r="I4" t="n">
         <v>78.59999999999999</v>
       </c>
-      <c r="I4" t="n">
+      <c r="J4" t="n">
         <v>4.45</v>
       </c>
-      <c r="J4" t="n">
+      <c r="K4" t="n">
         <v>1.64</v>
       </c>
-      <c r="K4" t="n">
+      <c r="L4" t="n">
         <v>7072</v>
       </c>
     </row>
@@ -971,11 +1004,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
     <col width="42" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
@@ -1007,35 +1041,40 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Corriente de fuga (mA)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Corriente Fase A (A)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Corriente Fase B (A)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Corriente Fase C (A)</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Potencia Activa (MW)</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Potencia Reactiva (MVAR)</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Num Operaciones</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Observacion</t>
         </is>
@@ -1062,21 +1101,24 @@
         <v>2.6</v>
       </c>
       <c r="F2" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="G2" t="n">
         <v>101.7</v>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>102.6</v>
       </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
         <v>103</v>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>5.67</v>
       </c>
-      <c r="J2" t="n">
+      <c r="K2" t="n">
         <v>2.32</v>
       </c>
-      <c r="K2" t="n">
+      <c r="L2" t="n">
         <v>11179</v>
       </c>
     </row>
@@ -1101,21 +1143,24 @@
         <v>2.9</v>
       </c>
       <c r="F3" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="G3" t="n">
         <v>97.8</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>96.2</v>
       </c>
-      <c r="H3" t="n">
+      <c r="I3" t="n">
         <v>97.5</v>
       </c>
-      <c r="I3" t="n">
+      <c r="J3" t="n">
         <v>5.19</v>
       </c>
-      <c r="J3" t="n">
+      <c r="K3" t="n">
         <v>2.61</v>
       </c>
-      <c r="K3" t="n">
+      <c r="L3" t="n">
         <v>7604</v>
       </c>
     </row>
@@ -1140,24 +1185,27 @@
         <v>5.5</v>
       </c>
       <c r="F4" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="G4" t="n">
         <v>112.1</v>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>110.3</v>
       </c>
-      <c r="H4" t="n">
+      <c r="I4" t="n">
         <v>112.3</v>
       </c>
-      <c r="I4" t="n">
+      <c r="J4" t="n">
         <v>6.06</v>
       </c>
-      <c r="J4" t="n">
+      <c r="K4" t="n">
         <v>2.79</v>
       </c>
-      <c r="K4" t="n">
+      <c r="L4" t="n">
         <v>3918</v>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>Tierra fuera de norma; revisar malla de puesta a tierra</t>
         </is>

</xml_diff>

<commit_message>
Completa equipos/subestaciones: hojas faltantes y nombre CTE-32L08
- Excel: renombrada hoja CTE-32L8 -> CTE-32L08 (coincide con el indice)
  y creadas las 15 hojas de datos faltantes (Coyoles Central, Bonito
  Oriental y nuevos interruptores/restauradores) con las columnas
  estandar + menu de cuadrilla. Hojas reordenadas como el indice.
- Ahora cargan los 18 equipos en 5 subestaciones.
- dashboard.py: los equipos sin visitas muestran un aviso en vez de
  graficos vacios.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Mantenimiento_Subestaciones.xlsx
+++ b/Mantenimiento_Subestaciones.xlsx
@@ -2,32 +2,51 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Equipos" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="CTE-32L8" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="CTE-32L08" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="SIS-32L30" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="ISL-32L44" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Limites" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="CTE-32L11" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="CTE-32L12" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="CTE-32L13" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="SIS-32L27" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="SIS-32L28" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="SIS-32L29" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="ISL-32L45" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="ISL-32L46" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="ISL-32L47" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="CCE-32L40" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="CCE-32L41" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="CCE-32L42" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="BOR-32L49" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="BOR-32L50" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="BOR-32L51" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="Limites" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
@@ -53,12 +72,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -421,12 +441,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:C19"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="2" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -454,12 +473,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CTE-32L8</t>
+          <t>CTE-32L08</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>interruptor</t>
+          <t>Interruptor</t>
         </is>
       </c>
     </row>
@@ -476,7 +495,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>restaurador</t>
+          <t>Restaurador</t>
         </is>
       </c>
     </row>
@@ -493,7 +512,262 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>restaurador</t>
+          <t>Restaurador</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Ceiba Termica</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>CTE-32L11</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Interruptor</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Ceiba Termica</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>CTE-32L12</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Interruptor</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Ceiba Termica</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>CTE-32L13</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Interruptor</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>San Isidro</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>SIS-32L27</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Interruptor</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>San Isidro</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>SIS-32L28</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Interruptor</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>San Isidro</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>SIS-32L29</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Interruptor</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Isletas</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ISL-32L45</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Restaurador</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Isletas</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ISL-32L46</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Restaurador</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Isletas</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ISL-32L47</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Restaurador</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Coyoles Central</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>CCE-32L40</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Restaurador</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Coyoles Central</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>CCE-32L41</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Restaurador</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Coyoles Central</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>CCE-32L42</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Restaurador</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Bonito Oriental</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>BOR-32L49</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Restaurador</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Bonito Oriental</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>BOR-32L50</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Restaurador</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Bonito Oriental</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>BOR-32L51</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Restaurador</t>
         </is>
       </c>
     </row>
@@ -510,6 +784,906 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Cuadrilla</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Voltaje VDC (V)</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Voltaje AC (V)</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Resistencia tierra (Ohm)</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente de fuga (mA)</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase A (A)</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase B (A)</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase C (A)</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Potencia Activa (MW)</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Potencia Reactiva (MVAR)</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Num Operaciones</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Observacion</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"LCB1,LCB2,TCO1"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Cuadrilla</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Voltaje VDC (V)</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Voltaje AC (V)</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Resistencia tierra (Ohm)</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente de fuga (mA)</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase A (A)</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase B (A)</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase C (A)</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Potencia Activa (MW)</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Potencia Reactiva (MVAR)</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Num Operaciones</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Observacion</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"LCB1,LCB2,TCO1"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Cuadrilla</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Voltaje VDC (V)</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Voltaje AC (V)</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Resistencia tierra (Ohm)</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente de fuga (mA)</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase A (A)</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase B (A)</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase C (A)</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Potencia Activa (MW)</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Potencia Reactiva (MVAR)</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Num Operaciones</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Observacion</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"LCB1,LCB2,TCO1"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Cuadrilla</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Voltaje VDC (V)</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Voltaje AC (V)</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Resistencia tierra (Ohm)</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente de fuga (mA)</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase A (A)</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase B (A)</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase C (A)</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Potencia Activa (MW)</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Potencia Reactiva (MVAR)</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Num Operaciones</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Observacion</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"LCB1,LCB2,TCO1"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Cuadrilla</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Voltaje VDC (V)</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Voltaje AC (V)</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Resistencia tierra (Ohm)</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente de fuga (mA)</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase A (A)</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase B (A)</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase C (A)</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Potencia Activa (MW)</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Potencia Reactiva (MVAR)</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Num Operaciones</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Observacion</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"LCB1,LCB2,TCO1"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Cuadrilla</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Voltaje VDC (V)</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Voltaje AC (V)</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Resistencia tierra (Ohm)</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente de fuga (mA)</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase A (A)</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase B (A)</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase C (A)</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Potencia Activa (MW)</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Potencia Reactiva (MVAR)</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Num Operaciones</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Observacion</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"LCB1,LCB2,TCO1"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Cuadrilla</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Voltaje VDC (V)</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Voltaje AC (V)</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Resistencia tierra (Ohm)</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente de fuga (mA)</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase A (A)</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase B (A)</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase C (A)</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Potencia Activa (MW)</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Potencia Reactiva (MVAR)</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Num Operaciones</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Observacion</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"LCB1,LCB2,TCO1"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Cuadrilla</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Voltaje VDC (V)</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Voltaje AC (V)</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Resistencia tierra (Ohm)</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente de fuga (mA)</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase A (A)</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase B (A)</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase C (A)</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Potencia Activa (MW)</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Potencia Reactiva (MVAR)</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Num Operaciones</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Observacion</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"LCB1,LCB2,TCO1"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Cuadrilla</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Voltaje VDC (V)</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Voltaje AC (V)</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Resistencia tierra (Ohm)</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente de fuga (mA)</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase A (A)</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase B (A)</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase C (A)</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Potencia Activa (MW)</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Potencia Reactiva (MVAR)</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Num Operaciones</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Observacion</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"LCB1,LCB2,TCO1"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Cuadrilla</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Voltaje VDC (V)</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Voltaje AC (V)</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Resistencia tierra (Ohm)</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente de fuga (mA)</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase A (A)</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase B (A)</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase C (A)</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Potencia Activa (MW)</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Potencia Reactiva (MVAR)</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Num Operaciones</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Observacion</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"LCB1,LCB2,TCO1"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -517,7 +1691,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -771,6 +1945,126 @@
       <formula1>"LCB2,TCO1,LCB1"</formula1>
     </dataValidation>
   </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Parametro</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Criterio</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Limite</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Regla</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Voltaje VDC</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>minimo</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>20</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>REVISAR si el valor es &lt;= 20</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Voltaje AC</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>minimo</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>119</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>REVISAR si el valor es &lt;= 119</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Resistencia tierra</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>maximo</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>5</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>REVISAR si el valor es &gt;= 5</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Ohm</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -782,7 +2076,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -1005,7 +2299,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -1227,116 +2521,446 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Parametro</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Criterio</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Limite</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Regla</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Unidad</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Voltaje VDC</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>minimo</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>20</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>REVISAR si el valor es &lt;= 20</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Voltaje AC</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>minimo</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>119</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>REVISAR si el valor es &lt;= 119</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Resistencia tierra</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>maximo</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>5</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>REVISAR si el valor es &gt;= 5</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Ohm</t>
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Cuadrilla</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Voltaje VDC (V)</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Voltaje AC (V)</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Resistencia tierra (Ohm)</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente de fuga (mA)</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase A (A)</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase B (A)</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase C (A)</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Potencia Activa (MW)</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Potencia Reactiva (MVAR)</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Num Operaciones</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Observacion</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"LCB1,LCB2,TCO1"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Cuadrilla</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Voltaje VDC (V)</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Voltaje AC (V)</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Resistencia tierra (Ohm)</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente de fuga (mA)</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase A (A)</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase B (A)</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase C (A)</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Potencia Activa (MW)</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Potencia Reactiva (MVAR)</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Num Operaciones</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Observacion</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"LCB1,LCB2,TCO1"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Cuadrilla</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Voltaje VDC (V)</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Voltaje AC (V)</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Resistencia tierra (Ohm)</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente de fuga (mA)</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase A (A)</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase B (A)</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase C (A)</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Potencia Activa (MW)</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Potencia Reactiva (MVAR)</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Num Operaciones</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Observacion</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"LCB1,LCB2,TCO1"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Cuadrilla</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Voltaje VDC (V)</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Voltaje AC (V)</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Resistencia tierra (Ohm)</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente de fuga (mA)</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase A (A)</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase B (A)</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase C (A)</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Potencia Activa (MW)</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Potencia Reactiva (MVAR)</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Num Operaciones</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Observacion</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"LCB1,LCB2,TCO1"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Cuadrilla</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Voltaje VDC (V)</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Voltaje AC (V)</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Resistencia tierra (Ohm)</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente de fuga (mA)</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase A (A)</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase B (A)</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase C (A)</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Potencia Activa (MW)</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Potencia Reactiva (MVAR)</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Num Operaciones</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Observacion</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"LCB1,LCB2,TCO1"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Ficha tecnica por equipo, subestacion Tela y correo sin graficos
- Excel: cada hoja de equipo lleva su FICHA TECNICA arriba (serie, marca,
  modelo, tipo, I nominal, tension, ano, ICC), leida de los formatos de
  Visita I. Agregada subestacion Tela (TEL-32L9, TEL-32L10, restauradores).
- modelos.Equipo.ficha; construir_modelo encuentra el encabezado de visitas
  dinamicamente y lee la ficha de las filas superiores.
- dashboard.py muestra la ficha tecnica por equipo (chips).
- agregar_equipo.py crea las hojas con el bloque de ficha.
- Correo (reporte_html) ya NO incluye graficos: solo motivo + ultima visita;
  los graficos quedan solo en el dashboard.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Mantenimiento_Subestaciones.xlsx
+++ b/Mantenimiento_Subestaciones.xlsx
@@ -25,7 +25,9 @@
     <sheet name="BOR-32L49" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="BOR-32L50" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="BOR-32L51" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="Limites" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="TEL-32L9" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="TEL-32L10" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Limites" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -441,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -766,6 +768,40 @@
         </is>
       </c>
       <c r="C19" t="inlineStr">
+        <is>
+          <t>Restaurador</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Tela</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>TEL-32L9</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Restaurador</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Tela</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>TEL-32L10</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
         <is>
           <t>Restaurador</t>
         </is>
@@ -790,83 +826,175 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
+          <t>FICHA TECNICA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Serie</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>A3255</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>SIEMENS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Modelo</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>8HH INTEMPERIE</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>I nominal (A)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>1250 A</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Tension</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>38 KV</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Ano</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2003</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>ICC</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>25 KA</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Cuadrilla</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Voltaje VDC (V)</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Voltaje AC (V)</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Resistencia tierra (Ohm)</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Corriente de fuga (mA)</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase A (A)</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase B (A)</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase C (A)</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>Potencia Activa (MW)</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>Potencia Reactiva (MVAR)</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>Num Operaciones</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>Observacion</t>
         </is>
       </c>
     </row>
+    <row r="8"/>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B8:B507" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"LCB1,LCB2,TCO1"</formula1>
     </dataValidation>
   </dataValidations>
@@ -880,83 +1008,173 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
+          <t>FICHA TECNICA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Serie</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>PR317020023</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ENTEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Modelo</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>EPR-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>I nominal (A)</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>800</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Tension</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>38 KV</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Ano</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>02/2017</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>ICC</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>16000 A</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Cuadrilla</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Voltaje VDC (V)</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Voltaje AC (V)</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Resistencia tierra (Ohm)</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Corriente de fuga (mA)</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase A (A)</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase B (A)</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase C (A)</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>Potencia Activa (MW)</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>Potencia Reactiva (MVAR)</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>Num Operaciones</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>Observacion</t>
         </is>
       </c>
     </row>
+    <row r="8"/>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B8:B507" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"LCB1,LCB2,TCO1"</formula1>
     </dataValidation>
   </dataValidations>
@@ -970,83 +1188,176 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
+          <t>FICHA TECNICA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Serie</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>PR318090566</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ENTEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Modelo</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ETR300-R600</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>EPR-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>I nominal (A)</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>800</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Tension</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>38 KV</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Ano</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>09/2018</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>ICC</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>16000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Cuadrilla</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Voltaje VDC (V)</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Voltaje AC (V)</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Resistencia tierra (Ohm)</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Corriente de fuga (mA)</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase A (A)</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase B (A)</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase C (A)</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>Potencia Activa (MW)</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>Potencia Reactiva (MVAR)</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>Num Operaciones</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>Observacion</t>
         </is>
       </c>
     </row>
+    <row r="8"/>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B8:B507" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"LCB1,LCB2,TCO1"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1060,83 +1371,171 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
+          <t>FICHA TECNICA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Serie</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>CP571102830-DB</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>COOPER</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Modelo</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>NOVA 38</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>I nominal (A)</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>630</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Tension</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>38 KV</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Ano</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>07/2007</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>ICC</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>12500</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Cuadrilla</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Voltaje VDC (V)</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Voltaje AC (V)</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Resistencia tierra (Ohm)</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Corriente de fuga (mA)</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase A (A)</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase B (A)</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase C (A)</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>Potencia Activa (MW)</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>Potencia Reactiva (MVAR)</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>Num Operaciones</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>Observacion</t>
         </is>
       </c>
     </row>
+    <row r="8"/>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B8:B507" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"LCB1,LCB2,TCO1"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1150,83 +1549,171 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
+          <t>FICHA TECNICA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Serie</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>PR318090562</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ENTEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Modelo</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>EPR-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>I nominal (A)</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>800</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Tension</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>38 KV</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Ano</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>09/2018</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>ICC</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>16000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Cuadrilla</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Voltaje VDC (V)</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Voltaje AC (V)</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Resistencia tierra (Ohm)</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Corriente de fuga (mA)</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase A (A)</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase B (A)</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase C (A)</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>Potencia Activa (MW)</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>Potencia Reactiva (MVAR)</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>Num Operaciones</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>Observacion</t>
         </is>
       </c>
     </row>
+    <row r="8"/>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B8:B507" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"LCB1,LCB2,TCO1"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1240,83 +1727,171 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
+          <t>FICHA TECNICA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Serie</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>S02B161VR3LH</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ABB</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Modelo</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>VR3S</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>I nominal (A)</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>800</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Tension</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>38 KV</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Ano</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>02/2002</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>ICC</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>16000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Cuadrilla</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Voltaje VDC (V)</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Voltaje AC (V)</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Resistencia tierra (Ohm)</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Corriente de fuga (mA)</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase A (A)</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase B (A)</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase C (A)</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>Potencia Activa (MW)</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>Potencia Reactiva (MVAR)</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>Num Operaciones</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>Observacion</t>
         </is>
       </c>
     </row>
+    <row r="8"/>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B8:B507" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"LCB1,LCB2,TCO1"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1330,83 +1905,171 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
+          <t>FICHA TECNICA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Serie</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>PR318090517</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ENTEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Modelo</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>EPR-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>I nominal (A)</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>800</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Tension</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>38 KV</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Ano</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>09/2018</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>ICC</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>16000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Cuadrilla</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Voltaje VDC (V)</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Voltaje AC (V)</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Resistencia tierra (Ohm)</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Corriente de fuga (mA)</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase A (A)</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase B (A)</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase C (A)</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>Potencia Activa (MW)</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>Potencia Reactiva (MVAR)</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>Num Operaciones</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>Observacion</t>
         </is>
       </c>
     </row>
+    <row r="8"/>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B8:B507" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"LCB1,LCB2,TCO1"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1420,83 +2083,140 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
+          <t>FICHA TECNICA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Serie</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Modelo</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>I nominal (A)</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Tension</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Ano</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>ICC</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Cuadrilla</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Voltaje VDC (V)</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Voltaje AC (V)</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Resistencia tierra (Ohm)</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Corriente de fuga (mA)</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase A (A)</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase B (A)</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase C (A)</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>Potencia Activa (MW)</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>Potencia Reactiva (MVAR)</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>Num Operaciones</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>Observacion</t>
         </is>
       </c>
     </row>
+    <row r="8"/>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B8:B507" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"LCB1,LCB2,TCO1"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1510,83 +2230,171 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
+          <t>FICHA TECNICA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Serie</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>PR318090514</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ENTEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Modelo</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>EPR-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>I nominal (A)</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>800</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Tension</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>38 KV</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Ano</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>09/2018</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>ICC</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>16000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Cuadrilla</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Voltaje VDC (V)</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Voltaje AC (V)</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Resistencia tierra (Ohm)</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Corriente de fuga (mA)</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase A (A)</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase B (A)</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase C (A)</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>Potencia Activa (MW)</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>Potencia Reactiva (MVAR)</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>Num Operaciones</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>Observacion</t>
         </is>
       </c>
     </row>
+    <row r="8"/>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B8:B507" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"LCB1,LCB2,TCO1"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1600,83 +2408,171 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
+          <t>FICHA TECNICA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Serie</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>CP571 423363</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>COOPER</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Modelo</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>NOVA 38</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>I nominal (A)</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>630</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Tension</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>38 KV</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Ano</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>06/2016</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>ICC</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>12500</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Cuadrilla</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Voltaje VDC (V)</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Voltaje AC (V)</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Resistencia tierra (Ohm)</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Corriente de fuga (mA)</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase A (A)</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase B (A)</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase C (A)</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>Potencia Activa (MW)</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>Potencia Reactiva (MVAR)</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>Num Operaciones</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>Observacion</t>
         </is>
       </c>
     </row>
+    <row r="8"/>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B8:B507" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"LCB1,LCB2,TCO1"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1690,250 +2586,337 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <dimension ref="A1:M11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="42" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>FICHA TECNICA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Serie</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>A-3250</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>SIEMENS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Modelo</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>8HH INTEMPERIE</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>I nominal (A)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>1250 A</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Tension</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>38 KV</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Ano</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2003</v>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>ICC</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>25 KA</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Cuadrilla</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Voltaje VDC (V)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Voltaje AC (V)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Resistencia tierra (Ohm)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Corriente de fuga (mA)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase A (A)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase B (A)</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase C (A)</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>Potencia Activa (MW)</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>Potencia Reactiva (MVAR)</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>Num Operaciones</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>Observacion</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>2025-09-16</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>LCB2</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="C8" t="n">
         <v>24.3</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D8" t="n">
         <v>121.2</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E8" t="n">
         <v>2.1</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F8" t="n">
         <v>4.4</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G8" t="n">
         <v>114.7</v>
       </c>
-      <c r="H2" t="n">
+      <c r="H8" t="n">
         <v>116.4</v>
       </c>
-      <c r="I2" t="n">
+      <c r="I8" t="n">
         <v>117.5</v>
       </c>
-      <c r="J2" t="n">
+      <c r="J8" t="n">
         <v>6.23</v>
       </c>
-      <c r="K2" t="n">
+      <c r="K8" t="n">
         <v>3.07</v>
       </c>
-      <c r="L2" t="n">
+      <c r="L8" t="n">
         <v>3408</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>2026-01-15</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>TCO1</t>
         </is>
       </c>
-      <c r="C3" t="n">
+      <c r="C9" t="n">
         <v>22</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D9" t="n">
         <v>121.7</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E9" t="n">
         <v>3.7</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F9" t="n">
         <v>6.8</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G9" t="n">
         <v>93.8</v>
       </c>
-      <c r="H3" t="n">
+      <c r="H9" t="n">
         <v>92.40000000000001</v>
       </c>
-      <c r="I3" t="n">
+      <c r="I9" t="n">
         <v>92.40000000000001</v>
       </c>
-      <c r="J3" t="n">
+      <c r="J9" t="n">
         <v>4.97</v>
       </c>
-      <c r="K3" t="n">
+      <c r="K9" t="n">
         <v>2.46</v>
       </c>
-      <c r="L3" t="n">
+      <c r="L9" t="n">
         <v>10711</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>2026-04-10</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>LCB1</t>
         </is>
       </c>
-      <c r="C4" t="n">
+      <c r="C10" t="n">
         <v>24.3</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D10" t="n">
         <v>121.3</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E10" t="n">
         <v>4.6</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F10" t="n">
         <v>8.5</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G10" t="n">
         <v>79</v>
       </c>
-      <c r="H4" t="n">
+      <c r="H10" t="n">
         <v>79.59999999999999</v>
       </c>
-      <c r="I4" t="n">
+      <c r="I10" t="n">
         <v>79.59999999999999</v>
       </c>
-      <c r="J4" t="n">
+      <c r="J10" t="n">
         <v>4.3</v>
       </c>
-      <c r="K4" t="n">
+      <c r="K10" t="n">
         <v>2</v>
       </c>
-      <c r="L4" t="n">
+      <c r="L10" t="n">
         <v>7737</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>2026-06-02</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>LCB2</t>
         </is>
       </c>
-      <c r="C5" t="n">
+      <c r="C11" t="n">
         <v>21.7</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D11" t="n">
         <v>122.3</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E11" t="n">
         <v>2.3</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F11" t="n">
         <v>4.7</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G11" t="n">
         <v>84.90000000000001</v>
       </c>
-      <c r="H5" t="n">
+      <c r="H11" t="n">
         <v>93.5</v>
       </c>
-      <c r="I5" t="n">
+      <c r="I11" t="n">
         <v>122.3</v>
       </c>
-      <c r="J5" t="n">
+      <c r="J11" t="n">
         <v>5.31</v>
       </c>
-      <c r="K5" t="n">
+      <c r="K11" t="n">
         <v>2.77</v>
       </c>
-      <c r="L5" t="n">
+      <c r="L11" t="n">
         <v>9359</v>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>Desbalance de corrientes entre fases</t>
         </is>
@@ -1941,8 +2924,8 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"LCB2,TCO1,LCB1"</formula1>
+    <dataValidation sqref="B8:B507" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"LCB1,LCB2,TCO1"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1950,6 +2933,370 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>FICHA TECNICA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Serie</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>CP571249416</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>COOPER</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Modelo</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>NOVA38</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>I nominal (A)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>630 A</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Tension</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>38 KV</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Ano</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>02/2011</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>ICC</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>12.5 KA</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Cuadrilla</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Voltaje VDC (V)</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Voltaje AC (V)</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Resistencia tierra (Ohm)</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Corriente de fuga (mA)</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase A (A)</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase B (A)</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase C (A)</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Potencia Activa (MW)</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Potencia Reactiva (MVAR)</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>Num Operaciones</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>Observacion</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="B8:B507" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"LCB1,LCB2,TCO1"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>FICHA TECNICA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Serie</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>PR317020024</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ENTEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Modelo</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>EPR-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>I nominal (A)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>800 A</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Tension</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>38 KV</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Ano</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>02/2017</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>ICC</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>16 KA</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Cuadrilla</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Voltaje VDC (V)</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Voltaje AC (V)</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Resistencia tierra (Ohm)</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Corriente de fuga (mA)</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase A (A)</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase B (A)</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Corriente Fase C (A)</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Potencia Activa (MW)</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Potencia Reactiva (MVAR)</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>Num Operaciones</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>Observacion</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="B8:B507" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"LCB1,LCB2,TCO1"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2075,217 +3422,297 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <dimension ref="A1:M10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="42" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>FICHA TECNICA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Serie</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ENTEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Modelo</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>EPR-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>I nominal (A)</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>800</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Tension</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>38 KV</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Ano</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>09/2018</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>ICC</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>16000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Cuadrilla</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Voltaje VDC (V)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Voltaje AC (V)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Resistencia tierra (Ohm)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Corriente de fuga (mA)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase A (A)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase B (A)</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase C (A)</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>Potencia Activa (MW)</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>Potencia Reactiva (MVAR)</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>Num Operaciones</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>Observacion</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>2025-10-05</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>LCB2</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="C8" t="n">
         <v>22.8</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D8" t="n">
         <v>120.7</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E8" t="n">
         <v>3.5</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F8" t="n">
         <v>6.4</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G8" t="n">
         <v>78.09999999999999</v>
       </c>
-      <c r="H2" t="n">
+      <c r="H8" t="n">
         <v>79</v>
       </c>
-      <c r="I2" t="n">
+      <c r="I8" t="n">
         <v>78.3</v>
       </c>
-      <c r="J2" t="n">
+      <c r="J8" t="n">
         <v>4.34</v>
       </c>
-      <c r="K2" t="n">
+      <c r="K8" t="n">
         <v>1.76</v>
       </c>
-      <c r="L2" t="n">
+      <c r="L8" t="n">
         <v>3013</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>2026-02-20</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>LCB2</t>
         </is>
       </c>
-      <c r="C3" t="n">
+      <c r="C9" t="n">
         <v>23.8</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D9" t="n">
         <v>121.4</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E9" t="n">
         <v>4.5</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F9" t="n">
         <v>7.9</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G9" t="n">
         <v>91.7</v>
       </c>
-      <c r="H3" t="n">
+      <c r="H9" t="n">
         <v>84.90000000000001</v>
       </c>
-      <c r="I3" t="n">
+      <c r="I9" t="n">
         <v>80.8</v>
       </c>
-      <c r="J3" t="n">
+      <c r="J9" t="n">
         <v>4.83</v>
       </c>
-      <c r="K3" t="n">
+      <c r="K9" t="n">
         <v>1.72</v>
       </c>
-      <c r="L3" t="n">
+      <c r="L9" t="n">
         <v>3341</v>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>Desbalance de corrientes entre fases</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>2026-06-02</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>TCO1</t>
         </is>
       </c>
-      <c r="C4" t="n">
+      <c r="C10" t="n">
         <v>23</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D10" t="n">
         <v>122.4</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E10" t="n">
         <v>2.2</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F10" t="n">
         <v>4.1</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G10" t="n">
         <v>79.09999999999999</v>
       </c>
-      <c r="H4" t="n">
+      <c r="H10" t="n">
         <v>80.2</v>
       </c>
-      <c r="I4" t="n">
+      <c r="I10" t="n">
         <v>78.59999999999999</v>
       </c>
-      <c r="J4" t="n">
+      <c r="J10" t="n">
         <v>4.45</v>
       </c>
-      <c r="K4" t="n">
+      <c r="K10" t="n">
         <v>1.64</v>
       </c>
-      <c r="L4" t="n">
+      <c r="L10" t="n">
         <v>7072</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"LCB2,TCO1,LCB1"</formula1>
+    <dataValidation sqref="B8:B507" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"LCB1,LCB2,TCO1"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2298,208 +3725,295 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <dimension ref="A1:M10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="42" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>FICHA TECNICA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Serie</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>PR318090568</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ENTEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Modelo</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>EPR-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>I nominal (A)</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>800</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Tension</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>38 KV</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Ano</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>09/2018</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>ICC</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>16000 A</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Cuadrilla</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Voltaje VDC (V)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Voltaje AC (V)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Resistencia tierra (Ohm)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Corriente de fuga (mA)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase A (A)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase B (A)</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase C (A)</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>Potencia Activa (MW)</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>Potencia Reactiva (MVAR)</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>Num Operaciones</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>Observacion</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>2025-11-12</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>TCO1</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="C8" t="n">
         <v>23.3</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D8" t="n">
         <v>120.1</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E8" t="n">
         <v>2.6</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F8" t="n">
         <v>5.2</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G8" t="n">
         <v>101.7</v>
       </c>
-      <c r="H2" t="n">
+      <c r="H8" t="n">
         <v>102.6</v>
       </c>
-      <c r="I2" t="n">
+      <c r="I8" t="n">
         <v>103</v>
       </c>
-      <c r="J2" t="n">
+      <c r="J8" t="n">
         <v>5.67</v>
       </c>
-      <c r="K2" t="n">
+      <c r="K8" t="n">
         <v>2.32</v>
       </c>
-      <c r="L2" t="n">
+      <c r="L8" t="n">
         <v>11179</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>2026-03-08</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>TCO1</t>
         </is>
       </c>
-      <c r="C3" t="n">
+      <c r="C9" t="n">
         <v>22.4</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D9" t="n">
         <v>121.5</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E9" t="n">
         <v>2.9</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F9" t="n">
         <v>5.7</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G9" t="n">
         <v>97.8</v>
       </c>
-      <c r="H3" t="n">
+      <c r="H9" t="n">
         <v>96.2</v>
       </c>
-      <c r="I3" t="n">
+      <c r="I9" t="n">
         <v>97.5</v>
       </c>
-      <c r="J3" t="n">
+      <c r="J9" t="n">
         <v>5.19</v>
       </c>
-      <c r="K3" t="n">
+      <c r="K9" t="n">
         <v>2.61</v>
       </c>
-      <c r="L3" t="n">
+      <c r="L9" t="n">
         <v>7604</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>2026-06-02</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>TCO1</t>
         </is>
       </c>
-      <c r="C4" t="n">
+      <c r="C10" t="n">
         <v>23.2</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D10" t="n">
         <v>122</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E10" t="n">
         <v>5.5</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F10" t="n">
         <v>9.6</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G10" t="n">
         <v>112.1</v>
       </c>
-      <c r="H4" t="n">
+      <c r="H10" t="n">
         <v>110.3</v>
       </c>
-      <c r="I4" t="n">
+      <c r="I10" t="n">
         <v>112.3</v>
       </c>
-      <c r="J4" t="n">
+      <c r="J10" t="n">
         <v>6.06</v>
       </c>
-      <c r="K4" t="n">
+      <c r="K10" t="n">
         <v>2.79</v>
       </c>
-      <c r="L4" t="n">
+      <c r="L10" t="n">
         <v>3918</v>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>Tierra fuera de norma; revisar malla de puesta a tierra</t>
         </is>
@@ -2507,8 +4021,8 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"LCB2,TCO1,LCB1"</formula1>
+    <dataValidation sqref="B8:B507" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"LCB1,LCB2,TCO1"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2521,83 +4035,173 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
+          <t>FICHA TECNICA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Serie</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>A-3248</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>SIEMENS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Modelo</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>8HH INTEMPERIE</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>I nominal (A)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>1250 A</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Tension</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>38 KV</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Ano</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2003</v>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>ICC</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>25 KA</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Cuadrilla</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Voltaje VDC (V)</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Voltaje AC (V)</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Resistencia tierra (Ohm)</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Corriente de fuga (mA)</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase A (A)</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase B (A)</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase C (A)</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>Potencia Activa (MW)</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>Potencia Reactiva (MVAR)</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>Num Operaciones</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>Observacion</t>
         </is>
       </c>
     </row>
+    <row r="8"/>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B8:B507" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"LCB1,LCB2,TCO1"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2611,83 +4215,173 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
+          <t>FICHA TECNICA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Serie</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>A-3253</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>SIEMENS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Modelo</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>8HH INTEMPERIE</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>I nominal (A)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>1250 A</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Tension</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>38 KV</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Ano</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2003</v>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>ICC</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>25 KA</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Cuadrilla</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Voltaje VDC (V)</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Voltaje AC (V)</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Resistencia tierra (Ohm)</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Corriente de fuga (mA)</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase A (A)</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase B (A)</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase C (A)</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>Potencia Activa (MW)</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>Potencia Reactiva (MVAR)</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>Num Operaciones</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>Observacion</t>
         </is>
       </c>
     </row>
+    <row r="8"/>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B8:B507" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"LCB1,LCB2,TCO1"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2701,83 +4395,175 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
+          <t>FICHA TECNICA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Serie</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>S01J139VB</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ABB</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Modelo</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>I nominal (A)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>1200 A</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Tension</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>38 KV</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Ano</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>09/2001</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>ICC</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>31500 A</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Cuadrilla</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Voltaje VDC (V)</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Voltaje AC (V)</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Resistencia tierra (Ohm)</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Corriente de fuga (mA)</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase A (A)</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase B (A)</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase C (A)</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>Potencia Activa (MW)</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>Potencia Reactiva (MVAR)</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>Num Operaciones</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>Observacion</t>
         </is>
       </c>
     </row>
+    <row r="8"/>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B8:B507" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"LCB1,LCB2,TCO1"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2791,83 +4577,175 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
+          <t>FICHA TECNICA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Serie</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>S02B118YB</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ABB</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Modelo</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>I nominal (A)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>1200 A</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Tension</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>38 KV</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Ano</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>02/2002</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>ICC</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>25 KA</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Cuadrilla</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Voltaje VDC (V)</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Voltaje AC (V)</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Resistencia tierra (Ohm)</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Corriente de fuga (mA)</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase A (A)</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase B (A)</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase C (A)</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>Potencia Activa (MW)</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>Potencia Reactiva (MVAR)</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>Num Operaciones</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>Observacion</t>
         </is>
       </c>
     </row>
+    <row r="8"/>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B8:B507" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"LCB1,LCB2,TCO1"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2881,83 +4759,175 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
+          <t>FICHA TECNICA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Serie</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1VAL09F118VB</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Marca</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ABB</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Modelo</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>BVRK</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>I nominal (A)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>1200 A</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Tension</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>38 KV</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Ano</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>07/2009</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>ICC</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>40 KA</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Cuadrilla</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Voltaje VDC (V)</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Voltaje AC (V)</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Resistencia tierra (Ohm)</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Corriente de fuga (mA)</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase A (A)</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase B (A)</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Corriente Fase C (A)</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>Potencia Activa (MW)</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>Potencia Reactiva (MVAR)</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>Num Operaciones</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>Observacion</t>
         </is>
       </c>
     </row>
+    <row r="8"/>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B8:B507" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"LCB1,LCB2,TCO1"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Datos sinteticos en 17 equipos, 5 alertas, enlace dashboard y enviar_historico
- Llena las 17 hojas de equipo vacias con visitas sinteticas (los 20 equipos ya tienen datos).
- Inyecta 5 alertas con tendencia para demo predictiva (2 tierra, 2 bajo VDC, 1 bajo VAC).
- Enlace al dashboard (config.DASHBOARD_URL) en correo y Telegram; vacio = no se muestra.
- Nuevo enviar_historico.py: envia el historico de N visitas de un equipo a destinatarios puntuales (--correo/--telegram/--demo).
- notificaciones: enviar_correo/enviar_telegram admiten destinatarios por llamada (override de config).
- README actualizado.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Mantenimiento_Subestaciones.xlsx
+++ b/Mantenimiento_Subestaciones.xlsx
@@ -826,7 +826,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -991,7 +991,132 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2025-10-31</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>LCB2</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>22.8</v>
+      </c>
+      <c r="D8" t="n">
+        <v>120.8</v>
+      </c>
+      <c r="E8" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="F8" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="G8" t="n">
+        <v>113.9</v>
+      </c>
+      <c r="H8" t="n">
+        <v>113.5</v>
+      </c>
+      <c r="I8" t="n">
+        <v>114</v>
+      </c>
+      <c r="J8" t="n">
+        <v>6.03</v>
+      </c>
+      <c r="K8" t="n">
+        <v>3.14</v>
+      </c>
+      <c r="L8" t="n">
+        <v>11096</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>LCB2</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>24</v>
+      </c>
+      <c r="D9" t="n">
+        <v>122.4</v>
+      </c>
+      <c r="E9" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="F9" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="G9" t="n">
+        <v>123.5</v>
+      </c>
+      <c r="H9" t="n">
+        <v>122.2</v>
+      </c>
+      <c r="I9" t="n">
+        <v>124.3</v>
+      </c>
+      <c r="J9" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="K9" t="n">
+        <v>2.84</v>
+      </c>
+      <c r="L9" t="n">
+        <v>5489</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>LCB1</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="D10" t="n">
+        <v>120.8</v>
+      </c>
+      <c r="E10" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="F10" t="n">
+        <v>5</v>
+      </c>
+      <c r="G10" t="n">
+        <v>102.3</v>
+      </c>
+      <c r="H10" t="n">
+        <v>104.3</v>
+      </c>
+      <c r="I10" t="n">
+        <v>103.8</v>
+      </c>
+      <c r="J10" t="n">
+        <v>5.62</v>
+      </c>
+      <c r="K10" t="n">
+        <v>2.58</v>
+      </c>
+      <c r="L10" t="n">
+        <v>6013</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="B8:B507" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -1008,7 +1133,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1171,7 +1296,132 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2025-11-25</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>LCB1</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>22.7</v>
+      </c>
+      <c r="D8" t="n">
+        <v>122.8</v>
+      </c>
+      <c r="E8" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F8" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="G8" t="n">
+        <v>111.6</v>
+      </c>
+      <c r="H8" t="n">
+        <v>113.5</v>
+      </c>
+      <c r="I8" t="n">
+        <v>113</v>
+      </c>
+      <c r="J8" t="n">
+        <v>6.02</v>
+      </c>
+      <c r="K8" t="n">
+        <v>3.02</v>
+      </c>
+      <c r="L8" t="n">
+        <v>3547</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-03-03</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>LCB2</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>22.7</v>
+      </c>
+      <c r="D9" t="n">
+        <v>120.7</v>
+      </c>
+      <c r="E9" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="F9" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="G9" t="n">
+        <v>96.8</v>
+      </c>
+      <c r="H9" t="n">
+        <v>95.2</v>
+      </c>
+      <c r="I9" t="n">
+        <v>93.5</v>
+      </c>
+      <c r="J9" t="n">
+        <v>5.03</v>
+      </c>
+      <c r="K9" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="L9" t="n">
+        <v>2876</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>LCB1</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>22.8</v>
+      </c>
+      <c r="D10" t="n">
+        <v>119.9</v>
+      </c>
+      <c r="E10" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F10" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="G10" t="n">
+        <v>117.8</v>
+      </c>
+      <c r="H10" t="n">
+        <v>118.2</v>
+      </c>
+      <c r="I10" t="n">
+        <v>118.4</v>
+      </c>
+      <c r="J10" t="n">
+        <v>6.23</v>
+      </c>
+      <c r="K10" t="n">
+        <v>3.32</v>
+      </c>
+      <c r="L10" t="n">
+        <v>9122</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="B8:B507" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -1188,7 +1438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1354,7 +1604,132 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2025-11-09</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>LCB2</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>22.3</v>
+      </c>
+      <c r="D8" t="n">
+        <v>120.9</v>
+      </c>
+      <c r="E8" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="F8" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="G8" t="n">
+        <v>88.2</v>
+      </c>
+      <c r="H8" t="n">
+        <v>86.7</v>
+      </c>
+      <c r="I8" t="n">
+        <v>88</v>
+      </c>
+      <c r="J8" t="n">
+        <v>4.84</v>
+      </c>
+      <c r="K8" t="n">
+        <v>2</v>
+      </c>
+      <c r="L8" t="n">
+        <v>7110</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-03-07</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>LCB2</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>23.7</v>
+      </c>
+      <c r="D9" t="n">
+        <v>120.6</v>
+      </c>
+      <c r="E9" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="F9" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="G9" t="n">
+        <v>80.5</v>
+      </c>
+      <c r="H9" t="n">
+        <v>82.40000000000001</v>
+      </c>
+      <c r="I9" t="n">
+        <v>81.3</v>
+      </c>
+      <c r="J9" t="n">
+        <v>4.36</v>
+      </c>
+      <c r="K9" t="n">
+        <v>2.16</v>
+      </c>
+      <c r="L9" t="n">
+        <v>11689</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>TCO1</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>22.1</v>
+      </c>
+      <c r="D10" t="n">
+        <v>123</v>
+      </c>
+      <c r="E10" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="F10" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G10" t="n">
+        <v>77.09999999999999</v>
+      </c>
+      <c r="H10" t="n">
+        <v>78</v>
+      </c>
+      <c r="I10" t="n">
+        <v>76.40000000000001</v>
+      </c>
+      <c r="J10" t="n">
+        <v>4.16</v>
+      </c>
+      <c r="K10" t="n">
+        <v>1.99</v>
+      </c>
+      <c r="L10" t="n">
+        <v>4569</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="B8:B507" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -1371,7 +1746,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1532,7 +1907,132 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2025-11-11</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>LCB2</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>23.9</v>
+      </c>
+      <c r="D8" t="n">
+        <v>120.2</v>
+      </c>
+      <c r="E8" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="F8" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G8" t="n">
+        <v>103.3</v>
+      </c>
+      <c r="H8" t="n">
+        <v>103</v>
+      </c>
+      <c r="I8" t="n">
+        <v>101.2</v>
+      </c>
+      <c r="J8" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="K8" t="n">
+        <v>2.89</v>
+      </c>
+      <c r="L8" t="n">
+        <v>11366</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-02-25</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>TCO1</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="D9" t="n">
+        <v>120.5</v>
+      </c>
+      <c r="E9" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="F9" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="G9" t="n">
+        <v>104.9</v>
+      </c>
+      <c r="H9" t="n">
+        <v>105.4</v>
+      </c>
+      <c r="I9" t="n">
+        <v>106.8</v>
+      </c>
+      <c r="J9" t="n">
+        <v>5.72</v>
+      </c>
+      <c r="K9" t="n">
+        <v>2.68</v>
+      </c>
+      <c r="L9" t="n">
+        <v>6845</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>LCB2</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="D10" t="n">
+        <v>121.4</v>
+      </c>
+      <c r="E10" t="n">
+        <v>4</v>
+      </c>
+      <c r="F10" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="G10" t="n">
+        <v>116</v>
+      </c>
+      <c r="H10" t="n">
+        <v>115.2</v>
+      </c>
+      <c r="I10" t="n">
+        <v>115.9</v>
+      </c>
+      <c r="J10" t="n">
+        <v>6.26</v>
+      </c>
+      <c r="K10" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="L10" t="n">
+        <v>4971</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="B8:B507" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -1549,7 +2049,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1710,7 +2210,137 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2025-11-14</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>LCB2</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="D8" t="n">
+        <v>121.2</v>
+      </c>
+      <c r="E8" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="F8" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="G8" t="n">
+        <v>119</v>
+      </c>
+      <c r="H8" t="n">
+        <v>118.3</v>
+      </c>
+      <c r="I8" t="n">
+        <v>119.5</v>
+      </c>
+      <c r="J8" t="n">
+        <v>6.43</v>
+      </c>
+      <c r="K8" t="n">
+        <v>3.03</v>
+      </c>
+      <c r="L8" t="n">
+        <v>2587</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-02-25</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>LCB1</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="D9" t="n">
+        <v>122.4</v>
+      </c>
+      <c r="E9" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="F9" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="G9" t="n">
+        <v>113.1</v>
+      </c>
+      <c r="H9" t="n">
+        <v>114.2</v>
+      </c>
+      <c r="I9" t="n">
+        <v>115.7</v>
+      </c>
+      <c r="J9" t="n">
+        <v>6.06</v>
+      </c>
+      <c r="K9" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="L9" t="n">
+        <v>4150</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>TCO1</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="D10" t="n">
+        <v>119.7</v>
+      </c>
+      <c r="E10" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="F10" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="G10" t="n">
+        <v>105.7</v>
+      </c>
+      <c r="H10" t="n">
+        <v>103.7</v>
+      </c>
+      <c r="I10" t="n">
+        <v>105.7</v>
+      </c>
+      <c r="J10" t="n">
+        <v>5.69</v>
+      </c>
+      <c r="K10" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="L10" t="n">
+        <v>5089</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Voltaje DC de control bajo (&lt;=20 V); revisar banco de baterias y cargador</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="B8:B507" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -1727,7 +2357,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1888,7 +2518,132 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2025-11-21</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>LCB1</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>22.8</v>
+      </c>
+      <c r="D8" t="n">
+        <v>122.1</v>
+      </c>
+      <c r="E8" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="F8" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="G8" t="n">
+        <v>119.4</v>
+      </c>
+      <c r="H8" t="n">
+        <v>119</v>
+      </c>
+      <c r="I8" t="n">
+        <v>119.7</v>
+      </c>
+      <c r="J8" t="n">
+        <v>6.63</v>
+      </c>
+      <c r="K8" t="n">
+        <v>2.63</v>
+      </c>
+      <c r="L8" t="n">
+        <v>2654</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-02-15</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>LCB2</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="D9" t="n">
+        <v>121.8</v>
+      </c>
+      <c r="E9" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="F9" t="n">
+        <v>9</v>
+      </c>
+      <c r="G9" t="n">
+        <v>115.4</v>
+      </c>
+      <c r="H9" t="n">
+        <v>113.8</v>
+      </c>
+      <c r="I9" t="n">
+        <v>114.7</v>
+      </c>
+      <c r="J9" t="n">
+        <v>6.04</v>
+      </c>
+      <c r="K9" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="L9" t="n">
+        <v>7655</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>LCB2</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>23.3</v>
+      </c>
+      <c r="D10" t="n">
+        <v>120.2</v>
+      </c>
+      <c r="E10" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="F10" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="G10" t="n">
+        <v>117</v>
+      </c>
+      <c r="H10" t="n">
+        <v>118.6</v>
+      </c>
+      <c r="I10" t="n">
+        <v>118.6</v>
+      </c>
+      <c r="J10" t="n">
+        <v>6.28</v>
+      </c>
+      <c r="K10" t="n">
+        <v>3.22</v>
+      </c>
+      <c r="L10" t="n">
+        <v>5026</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="B8:B507" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -1905,7 +2660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2066,7 +2821,132 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2025-11-27</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>LCB1</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="D8" t="n">
+        <v>122.1</v>
+      </c>
+      <c r="E8" t="n">
+        <v>3</v>
+      </c>
+      <c r="F8" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="G8" t="n">
+        <v>108.4</v>
+      </c>
+      <c r="H8" t="n">
+        <v>106.4</v>
+      </c>
+      <c r="I8" t="n">
+        <v>107.4</v>
+      </c>
+      <c r="J8" t="n">
+        <v>5.91</v>
+      </c>
+      <c r="K8" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="L8" t="n">
+        <v>9970</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>TCO1</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="D9" t="n">
+        <v>120.8</v>
+      </c>
+      <c r="E9" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="F9" t="n">
+        <v>5</v>
+      </c>
+      <c r="G9" t="n">
+        <v>114.3</v>
+      </c>
+      <c r="H9" t="n">
+        <v>116.2</v>
+      </c>
+      <c r="I9" t="n">
+        <v>113.8</v>
+      </c>
+      <c r="J9" t="n">
+        <v>6.18</v>
+      </c>
+      <c r="K9" t="n">
+        <v>2.97</v>
+      </c>
+      <c r="L9" t="n">
+        <v>11700</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>LCB2</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>22.8</v>
+      </c>
+      <c r="D10" t="n">
+        <v>122.7</v>
+      </c>
+      <c r="E10" t="n">
+        <v>4</v>
+      </c>
+      <c r="F10" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="G10" t="n">
+        <v>95.7</v>
+      </c>
+      <c r="H10" t="n">
+        <v>94.7</v>
+      </c>
+      <c r="I10" t="n">
+        <v>95.5</v>
+      </c>
+      <c r="J10" t="n">
+        <v>5.11</v>
+      </c>
+      <c r="K10" t="n">
+        <v>2.51</v>
+      </c>
+      <c r="L10" t="n">
+        <v>8236</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="B8:B507" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -2083,7 +2963,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2213,7 +3093,132 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2025-11-15</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>LCB1</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="D8" t="n">
+        <v>121.1</v>
+      </c>
+      <c r="E8" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="F8" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="G8" t="n">
+        <v>87.40000000000001</v>
+      </c>
+      <c r="H8" t="n">
+        <v>88.5</v>
+      </c>
+      <c r="I8" t="n">
+        <v>87.40000000000001</v>
+      </c>
+      <c r="J8" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="K8" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="L8" t="n">
+        <v>4850</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-03-12</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>LCB2</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="D9" t="n">
+        <v>120</v>
+      </c>
+      <c r="E9" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="F9" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="G9" t="n">
+        <v>95.3</v>
+      </c>
+      <c r="H9" t="n">
+        <v>95.2</v>
+      </c>
+      <c r="I9" t="n">
+        <v>94.90000000000001</v>
+      </c>
+      <c r="J9" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="K9" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="L9" t="n">
+        <v>10604</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>LCB2</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="D10" t="n">
+        <v>122.5</v>
+      </c>
+      <c r="E10" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="F10" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="G10" t="n">
+        <v>102</v>
+      </c>
+      <c r="H10" t="n">
+        <v>102</v>
+      </c>
+      <c r="I10" t="n">
+        <v>103.1</v>
+      </c>
+      <c r="J10" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="K10" t="n">
+        <v>2.46</v>
+      </c>
+      <c r="L10" t="n">
+        <v>2672</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="B8:B507" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -2230,7 +3235,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2391,7 +3396,132 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2025-11-06</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>LCB1</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="D8" t="n">
+        <v>122.3</v>
+      </c>
+      <c r="E8" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="F8" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="G8" t="n">
+        <v>76</v>
+      </c>
+      <c r="H8" t="n">
+        <v>76.09999999999999</v>
+      </c>
+      <c r="I8" t="n">
+        <v>76.90000000000001</v>
+      </c>
+      <c r="J8" t="n">
+        <v>4.09</v>
+      </c>
+      <c r="K8" t="n">
+        <v>2.02</v>
+      </c>
+      <c r="L8" t="n">
+        <v>5927</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>LCB2</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>24</v>
+      </c>
+      <c r="D9" t="n">
+        <v>121.4</v>
+      </c>
+      <c r="E9" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="F9" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="G9" t="n">
+        <v>103.3</v>
+      </c>
+      <c r="H9" t="n">
+        <v>103.7</v>
+      </c>
+      <c r="I9" t="n">
+        <v>102.2</v>
+      </c>
+      <c r="J9" t="n">
+        <v>5.72</v>
+      </c>
+      <c r="K9" t="n">
+        <v>2.28</v>
+      </c>
+      <c r="L9" t="n">
+        <v>10093</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>LCB2</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="D10" t="n">
+        <v>121.9</v>
+      </c>
+      <c r="E10" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="F10" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="G10" t="n">
+        <v>96.09999999999999</v>
+      </c>
+      <c r="H10" t="n">
+        <v>94.8</v>
+      </c>
+      <c r="I10" t="n">
+        <v>94.5</v>
+      </c>
+      <c r="J10" t="n">
+        <v>5.27</v>
+      </c>
+      <c r="K10" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="L10" t="n">
+        <v>3228</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="B8:B507" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -2408,7 +3538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2569,7 +3699,137 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2025-10-31</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>TCO1</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="D8" t="n">
+        <v>120.8</v>
+      </c>
+      <c r="E8" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F8" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="G8" t="n">
+        <v>89.09999999999999</v>
+      </c>
+      <c r="H8" t="n">
+        <v>85.90000000000001</v>
+      </c>
+      <c r="I8" t="n">
+        <v>87.7</v>
+      </c>
+      <c r="J8" t="n">
+        <v>4.61</v>
+      </c>
+      <c r="K8" t="n">
+        <v>2.48</v>
+      </c>
+      <c r="L8" t="n">
+        <v>8499</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>TCO1</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="D9" t="n">
+        <v>122.2</v>
+      </c>
+      <c r="E9" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="F9" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="G9" t="n">
+        <v>116.3</v>
+      </c>
+      <c r="H9" t="n">
+        <v>115.8</v>
+      </c>
+      <c r="I9" t="n">
+        <v>116.8</v>
+      </c>
+      <c r="J9" t="n">
+        <v>6.14</v>
+      </c>
+      <c r="K9" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="L9" t="n">
+        <v>10838</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>TCO1</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>23.7</v>
+      </c>
+      <c r="D10" t="n">
+        <v>122.2</v>
+      </c>
+      <c r="E10" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="F10" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="G10" t="n">
+        <v>79.59999999999999</v>
+      </c>
+      <c r="H10" t="n">
+        <v>79.09999999999999</v>
+      </c>
+      <c r="I10" t="n">
+        <v>79.09999999999999</v>
+      </c>
+      <c r="J10" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="K10" t="n">
+        <v>2.09</v>
+      </c>
+      <c r="L10" t="n">
+        <v>5468</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Resistencia de tierra fuera de norma (&gt;=5 Ohm); revisar malla de puesta a tierra</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="B8:B507" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -2938,7 +4198,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3103,7 +4363,137 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2025-10-24</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>TCO1</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>23.3</v>
+      </c>
+      <c r="D8" t="n">
+        <v>121.4</v>
+      </c>
+      <c r="E8" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="F8" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="G8" t="n">
+        <v>123.6</v>
+      </c>
+      <c r="H8" t="n">
+        <v>123.9</v>
+      </c>
+      <c r="I8" t="n">
+        <v>124.5</v>
+      </c>
+      <c r="J8" t="n">
+        <v>6.57</v>
+      </c>
+      <c r="K8" t="n">
+        <v>3.43</v>
+      </c>
+      <c r="L8" t="n">
+        <v>5961</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-02-16</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>TCO1</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>24</v>
+      </c>
+      <c r="D9" t="n">
+        <v>120.1</v>
+      </c>
+      <c r="E9" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="F9" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="G9" t="n">
+        <v>102.2</v>
+      </c>
+      <c r="H9" t="n">
+        <v>105.2</v>
+      </c>
+      <c r="I9" t="n">
+        <v>102.5</v>
+      </c>
+      <c r="J9" t="n">
+        <v>5.62</v>
+      </c>
+      <c r="K9" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="L9" t="n">
+        <v>11332</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>TCO1</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="D10" t="n">
+        <v>118.4</v>
+      </c>
+      <c r="E10" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="F10" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="G10" t="n">
+        <v>83.2</v>
+      </c>
+      <c r="H10" t="n">
+        <v>82.5</v>
+      </c>
+      <c r="I10" t="n">
+        <v>83.2</v>
+      </c>
+      <c r="J10" t="n">
+        <v>4.58</v>
+      </c>
+      <c r="K10" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="L10" t="n">
+        <v>7093</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Voltaje AC de servicios propios bajo (&lt;=119 V); revisar alimentacion de servicios auxiliares</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="B8:B507" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -3120,7 +4510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3285,7 +4675,132 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2025-11-08</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>LCB1</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>23.1</v>
+      </c>
+      <c r="D8" t="n">
+        <v>120.2</v>
+      </c>
+      <c r="E8" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="F8" t="n">
+        <v>4</v>
+      </c>
+      <c r="G8" t="n">
+        <v>82.7</v>
+      </c>
+      <c r="H8" t="n">
+        <v>82.8</v>
+      </c>
+      <c r="I8" t="n">
+        <v>81.3</v>
+      </c>
+      <c r="J8" t="n">
+        <v>4.38</v>
+      </c>
+      <c r="K8" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="L8" t="n">
+        <v>8466</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>LCB2</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="D9" t="n">
+        <v>119.9</v>
+      </c>
+      <c r="E9" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="F9" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="G9" t="n">
+        <v>120</v>
+      </c>
+      <c r="H9" t="n">
+        <v>120</v>
+      </c>
+      <c r="I9" t="n">
+        <v>119.2</v>
+      </c>
+      <c r="J9" t="n">
+        <v>6.42</v>
+      </c>
+      <c r="K9" t="n">
+        <v>3.16</v>
+      </c>
+      <c r="L9" t="n">
+        <v>6714</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>LCB2</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>22.8</v>
+      </c>
+      <c r="D10" t="n">
+        <v>119.7</v>
+      </c>
+      <c r="E10" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="F10" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="G10" t="n">
+        <v>78.59999999999999</v>
+      </c>
+      <c r="H10" t="n">
+        <v>80.5</v>
+      </c>
+      <c r="I10" t="n">
+        <v>78.8</v>
+      </c>
+      <c r="J10" t="n">
+        <v>4.33</v>
+      </c>
+      <c r="K10" t="n">
+        <v>1.93</v>
+      </c>
+      <c r="L10" t="n">
+        <v>10602</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="B8:B507" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -4035,7 +5550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4198,7 +5713,137 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2025-10-27</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>TCO1</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="D8" t="n">
+        <v>122.6</v>
+      </c>
+      <c r="E8" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="F8" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="G8" t="n">
+        <v>104.9</v>
+      </c>
+      <c r="H8" t="n">
+        <v>103.6</v>
+      </c>
+      <c r="I8" t="n">
+        <v>104.9</v>
+      </c>
+      <c r="J8" t="n">
+        <v>5.63</v>
+      </c>
+      <c r="K8" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="L8" t="n">
+        <v>2541</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>LCB2</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="D9" t="n">
+        <v>120</v>
+      </c>
+      <c r="E9" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="F9" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="G9" t="n">
+        <v>116.5</v>
+      </c>
+      <c r="H9" t="n">
+        <v>114.5</v>
+      </c>
+      <c r="I9" t="n">
+        <v>114.7</v>
+      </c>
+      <c r="J9" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="K9" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="L9" t="n">
+        <v>8343</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>TCO1</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>24</v>
+      </c>
+      <c r="D10" t="n">
+        <v>123</v>
+      </c>
+      <c r="E10" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="F10" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="G10" t="n">
+        <v>91.40000000000001</v>
+      </c>
+      <c r="H10" t="n">
+        <v>91.90000000000001</v>
+      </c>
+      <c r="I10" t="n">
+        <v>93.09999999999999</v>
+      </c>
+      <c r="J10" t="n">
+        <v>5.04</v>
+      </c>
+      <c r="K10" t="n">
+        <v>2.22</v>
+      </c>
+      <c r="L10" t="n">
+        <v>11960</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Resistencia de tierra fuera de norma (&gt;=5 Ohm); revisar malla de puesta a tierra</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="B8:B507" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -4215,7 +5860,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4378,7 +6023,132 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2025-11-08</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>LCB2</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="D8" t="n">
+        <v>121.3</v>
+      </c>
+      <c r="E8" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="F8" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="G8" t="n">
+        <v>112.5</v>
+      </c>
+      <c r="H8" t="n">
+        <v>114.1</v>
+      </c>
+      <c r="I8" t="n">
+        <v>111.6</v>
+      </c>
+      <c r="J8" t="n">
+        <v>6.07</v>
+      </c>
+      <c r="K8" t="n">
+        <v>2.92</v>
+      </c>
+      <c r="L8" t="n">
+        <v>10351</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>LCB2</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>23.3</v>
+      </c>
+      <c r="D9" t="n">
+        <v>122.3</v>
+      </c>
+      <c r="E9" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="F9" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="G9" t="n">
+        <v>116</v>
+      </c>
+      <c r="H9" t="n">
+        <v>116.9</v>
+      </c>
+      <c r="I9" t="n">
+        <v>117.1</v>
+      </c>
+      <c r="J9" t="n">
+        <v>6.28</v>
+      </c>
+      <c r="K9" t="n">
+        <v>3.03</v>
+      </c>
+      <c r="L9" t="n">
+        <v>4833</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>LCB2</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="D10" t="n">
+        <v>120.4</v>
+      </c>
+      <c r="E10" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="F10" t="n">
+        <v>9</v>
+      </c>
+      <c r="G10" t="n">
+        <v>99</v>
+      </c>
+      <c r="H10" t="n">
+        <v>99.2</v>
+      </c>
+      <c r="I10" t="n">
+        <v>98</v>
+      </c>
+      <c r="J10" t="n">
+        <v>5.36</v>
+      </c>
+      <c r="K10" t="n">
+        <v>2.47</v>
+      </c>
+      <c r="L10" t="n">
+        <v>7540</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="B8:B507" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -4395,7 +6165,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4560,7 +6330,132 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2025-11-24</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>TCO1</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="D8" t="n">
+        <v>119.6</v>
+      </c>
+      <c r="E8" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="F8" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="G8" t="n">
+        <v>125.2</v>
+      </c>
+      <c r="H8" t="n">
+        <v>122.3</v>
+      </c>
+      <c r="I8" t="n">
+        <v>121.5</v>
+      </c>
+      <c r="J8" t="n">
+        <v>6.72</v>
+      </c>
+      <c r="K8" t="n">
+        <v>2.98</v>
+      </c>
+      <c r="L8" t="n">
+        <v>10145</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>LCB2</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>23.3</v>
+      </c>
+      <c r="D9" t="n">
+        <v>122.4</v>
+      </c>
+      <c r="E9" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="F9" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="G9" t="n">
+        <v>119.4</v>
+      </c>
+      <c r="H9" t="n">
+        <v>122.5</v>
+      </c>
+      <c r="I9" t="n">
+        <v>118.3</v>
+      </c>
+      <c r="J9" t="n">
+        <v>6.56</v>
+      </c>
+      <c r="K9" t="n">
+        <v>2.91</v>
+      </c>
+      <c r="L9" t="n">
+        <v>10940</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>LCB1</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="D10" t="n">
+        <v>122.7</v>
+      </c>
+      <c r="E10" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F10" t="n">
+        <v>5</v>
+      </c>
+      <c r="G10" t="n">
+        <v>112.2</v>
+      </c>
+      <c r="H10" t="n">
+        <v>113.5</v>
+      </c>
+      <c r="I10" t="n">
+        <v>110.7</v>
+      </c>
+      <c r="J10" t="n">
+        <v>5.96</v>
+      </c>
+      <c r="K10" t="n">
+        <v>3.06</v>
+      </c>
+      <c r="L10" t="n">
+        <v>9238</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="B8:B507" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -4577,7 +6472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4742,7 +6637,137 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2025-10-29</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>LCB1</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="D8" t="n">
+        <v>121.7</v>
+      </c>
+      <c r="E8" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F8" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="G8" t="n">
+        <v>76.7</v>
+      </c>
+      <c r="H8" t="n">
+        <v>77.90000000000001</v>
+      </c>
+      <c r="I8" t="n">
+        <v>76.90000000000001</v>
+      </c>
+      <c r="J8" t="n">
+        <v>4.06</v>
+      </c>
+      <c r="K8" t="n">
+        <v>2.19</v>
+      </c>
+      <c r="L8" t="n">
+        <v>11909</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-02-14</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>LCB2</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="D9" t="n">
+        <v>122.8</v>
+      </c>
+      <c r="E9" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="F9" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="G9" t="n">
+        <v>81.90000000000001</v>
+      </c>
+      <c r="H9" t="n">
+        <v>82.5</v>
+      </c>
+      <c r="I9" t="n">
+        <v>82.3</v>
+      </c>
+      <c r="J9" t="n">
+        <v>4.45</v>
+      </c>
+      <c r="K9" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="L9" t="n">
+        <v>3883</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>LCB2</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="D10" t="n">
+        <v>120.1</v>
+      </c>
+      <c r="E10" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="F10" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="G10" t="n">
+        <v>104</v>
+      </c>
+      <c r="H10" t="n">
+        <v>103.2</v>
+      </c>
+      <c r="I10" t="n">
+        <v>105.3</v>
+      </c>
+      <c r="J10" t="n">
+        <v>5.59</v>
+      </c>
+      <c r="K10" t="n">
+        <v>2.74</v>
+      </c>
+      <c r="L10" t="n">
+        <v>4238</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Voltaje DC de control bajo (&lt;=20 V); revisar banco de baterias y cargador</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="B8:B507" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -4759,7 +6784,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4924,7 +6949,132 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2025-11-13</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>TCO1</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="D8" t="n">
+        <v>119.7</v>
+      </c>
+      <c r="E8" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="F8" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="G8" t="n">
+        <v>97.5</v>
+      </c>
+      <c r="H8" t="n">
+        <v>97.40000000000001</v>
+      </c>
+      <c r="I8" t="n">
+        <v>98</v>
+      </c>
+      <c r="J8" t="n">
+        <v>5.18</v>
+      </c>
+      <c r="K8" t="n">
+        <v>2.68</v>
+      </c>
+      <c r="L8" t="n">
+        <v>11013</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>LCB2</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="D9" t="n">
+        <v>121.7</v>
+      </c>
+      <c r="E9" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="F9" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="G9" t="n">
+        <v>108.9</v>
+      </c>
+      <c r="H9" t="n">
+        <v>111.1</v>
+      </c>
+      <c r="I9" t="n">
+        <v>109.4</v>
+      </c>
+      <c r="J9" t="n">
+        <v>5.99</v>
+      </c>
+      <c r="K9" t="n">
+        <v>2.68</v>
+      </c>
+      <c r="L9" t="n">
+        <v>3289</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>TCO1</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>23.1</v>
+      </c>
+      <c r="D10" t="n">
+        <v>122.2</v>
+      </c>
+      <c r="E10" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F10" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="G10" t="n">
+        <v>118.9</v>
+      </c>
+      <c r="H10" t="n">
+        <v>119.4</v>
+      </c>
+      <c r="I10" t="n">
+        <v>118.9</v>
+      </c>
+      <c r="J10" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="K10" t="n">
+        <v>2.66</v>
+      </c>
+      <c r="L10" t="n">
+        <v>5127</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="B8:B507" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">

</xml_diff>